<commit_message>
feat(US01): bổ sung 7 TC review gaps + cập nhật chuẩn URD_Ref trong skill
- Test_Cases_US01.xlsx: bổ sung 7 TC mới từ kết quả review (GAP-01~07)
  - US01-BR-NEG-012: Chỉnh sửa NV - Tên/Mô tả read-only
  - US01-BR-NEG-013: Sửa HHLực NV < HHLực SPDV con (Critical)
  - US01-BR-HAP-013: Batch - T trong khoảng [HLực,HHLực] không đổi trạng thái
  - US01-BR-HAP-014: Sửa SPDV chi tiết happy path (Critical)
  - US01-BR-NEG-014: Sửa SPDV chi tiết vi phạm ngày cha (Critical)
  - US01-BR-HAP-015: BVA last-valid Mã 99
  - US01-BR-NEG-015: Bỏ trống Mô tả (pending BA confirm)
  - Tổng TC: 33 → 40 | Critical: 12→15 | High: 17→19 | Medium: 4→6

- qa_test_case_generator/SKILL.md: nâng chuẩn cột URD_Ref (section 7.2)
  - Thêm cấu trúc bắt buộc 2 phần: [Vị trí] – [Trích dẫn ≤30 từ]
  - Bổ sung bảng ví dụ 5 loại trường hợp thực tế

- Xóa script tạm generate_us01_testcases.py (cleanup)
</commit_message>
<xml_diff>
--- a/Feature_02_SA_Tham_So_He_Thong/test-cases/Test_Cases_US01.xlsx
+++ b/Feature_02_SA_Tham_So_He_Thong/test-cases/Test_Cases_US01.xlsx
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U34"/>
+  <dimension ref="A1:U41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3430,6 +3430,574 @@
       <c r="T34" s="4" t="inlineStr"/>
       <c r="U34" s="4" t="inlineStr"/>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>US01-BR-NEG-012</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>LOG-NV-EDIT-RESTRICT</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Mục "Khai báo Nghiệp vụ" - P15: "hệ thống chỉ cho phép chỉnh sửa Ngày hiệu lực, Ngày hết hiệu lực"</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>SA - Tham Số Hệ Thống</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Khai báo Danh mục Sản phẩm Dịch vụ và Code Phí</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Chỉnh sửa Nghiệp vụ – Các trường Tên NV và Mô tả hiển thị read-only, không thể chỉnh sửa</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>TC-BR</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>1. Nghiệp vụ 'Bảo Lãnh' (Mã '02') đã duyệt thành công, Trạng thái = Hoạt động.
+2. Đã đăng nhập với tài khoản Maker có quyền 'Danh mục Sản phẩm Dịch vụ và Code Phí'.
+3. Ngày hệ thống (T) = 21/04/2026.</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>1. Truy cập menu: Tham số &gt;&gt; Danh mục sản phẩm dịch vụ và Code phí.
+2. Tại dòng 'Bảo Lãnh' (Mã '02'), nhấn nút 'Chỉnh sửa'.
+3. Quan sát trạng thái các trường trên màn hình Chỉnh sửa: Mã NV, Tên NV, Mô tả.
+4. Thử nhấn vào trường 'Tên NV' và nhập ký tự bất kỳ.
+5. Thử nhấn vào trường 'Mô tả' và nhập ký tự bất kỳ.</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>(i) Nghiệp vụ/Logic: Hệ thống chỉ cho phép chỉnh sửa Ngày hiệu lực và Ngày hết hiệu lực. Các trường còn lại bị khóa.
+(ii) UI: Trường 'Mã NV', 'Tên NV', 'Mô tả' hiển thị ở chế độ read-only (disabled/không có input cursor). Không thể nhập ký tự vào các trường này. Chỉ trường 'Ngày hiệu lực' và 'Ngày hết hiệu lực' cho phép chỉnh sửa.
+(iii) Trạng thái bản ghi: Không thay đổi (chưa nhấn Xác nhận).
+(iv) Output: Không.</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>US01-NV-EDIT-READONLY</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Review GAP-02: Xác nhận UX theo Q14 BA confirm "màn hình chỉnh sửa tương tự màn hình xem chi tiết nhưng chỉnh sửa được một số trường".</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>US01-BR-NEG-013</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>LOG-NV-EDIT-CASCADE</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Mục "Khai báo Nghiệp vụ" - P17: "Ngày hết hiệu lực phải &gt;= Ngày hết hiệu lực của các SPDV chi tiết"</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>SA - Tham Số Hệ Thống</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Khai báo Danh mục Sản phẩm Dịch vụ và Code Phí</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Chỉnh sửa Nghiệp vụ thất bại – Ngày hết hiệu lực mới nhỏ hơn Ngày hết hiệu lực của SPDV con</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>TC-BR</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>1. Nghiệp vụ 'Tài Khoản' (Mã '01') đã duyệt: Ngày HLực = 01/04/2026; Ngày HHLực = 31/12/2027.
+2. SPDV con '0101 - TK Thanh Toán' đã duyệt: Ngày HLực = 01/04/2026; Ngày HHLực = 30/11/2027.
+3. Đã đăng nhập Maker. Ngày hệ thống (T) = 21/04/2026.</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>1. Truy cập menu: Tham số &gt;&gt; Danh mục sản phẩm dịch vụ và Code phí.
+2. Tại dòng 'Tài Khoản' (Mã '01'), nhấn 'Chỉnh sửa'.
+3. Sửa Ngày hết hiệu lực từ 31/12/2027 → 31/10/2027 (nhỏ hơn HHLực của '0101' = 30/11/2027).
+4. Giữ nguyên Ngày hiệu lực = 01/04/2026.
+5. Nhấn 'Xác nhận'.</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>(i) Nghiệp vụ/Logic: Hệ thống từ chối vì Ngày HHLực mới (31/10/2027) &lt; Ngày HHLực của SPDV con '0101' (30/11/2027). Vi phạm ràng buộc P17.
+(ii) UI: Hiển thị thông báo lỗi tại trường Ngày hết hiệu lực: 'Ngày hết hiệu lực phải lớn hơn hoặc bằng Ngày hết hiệu lực của SPDV chi tiết con (30/11/2027)'. Form vẫn mở, giữ nguyên dữ liệu.
+(iii) Trạng thái bản ghi: Không tạo bản ghi Pending mới. Nghiệp vụ 'Tài Khoản' giữ nguyên HHLực = 31/12/2027.
+(iv) Output: Không.</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>US01-NV-EDIT-HHLUCC-VIOLATION</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Review GAP-03: Bổ sung chiều HHLực bị thiếu trong NEG-007. Track Q12 – cần verify lại khi BA update US.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>US01-BR-HAP-013</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>LOG-NV-BATCH-JOB</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Mục "Khai báo Nghiệp vụ" - P20-P21: Batch đầu ngày cập nhật trạng thái</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>SA - Tham Số Hệ Thống</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Khai báo Danh mục Sản phẩm Dịch vụ và Code Phí</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Auto-Job đầu ngày – Nghiệp vụ đang Hoạt động, ngày T nằm trong khoảng [HLực, HHLực]: trạng thái không thay đổi</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>TC-BR</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>1. Nghiệp vụ 'Ngoại Hối' (Mã '04') đã duyệt, Trạng thái = Hoạt động.
+   Ngày hiệu lực = 01/04/2026; Ngày hết hiệu lực = 31/12/2026.
+2. Ngày hệ thống (T) = 21/04/2026 (nằm trong khoảng [01/04/2026, 31/12/2026]).
+3. Batch Job đầu ngày đã được trigger/chạy.</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>1. Trigger Batch Job đầu ngày (mock system date = 21/04/2026 hoặc chạy thủ công trên môi trường test).
+2. Sau khi Batch chạy xong, truy cập màn hình Danh mục SPDV.
+3. Kiểm tra trạng thái Nghiệp vụ 'Ngoại Hối' (Mã '04').</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>(i) Nghiệp vụ/Logic: Vì ngày T (21/04/2026) nằm trong khoảng [HLực=01/04/2026, HHLực=31/12/2026], không có điều kiện nào trong P20/P21 được kích hoạt. Trạng thái giữ nguyên = Hoạt động.
+(ii) UI: Cột Trạng thái của 'Ngoại Hối' hiển thị 'Hoạt động' (không thay đổi).
+(iii) Trạng thái bản ghi: Bản ghi không bị cập nhật bởi Batch Job.
+(iv) Output: Không.</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>US01-BATCH-NO-CHANGE</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Review GAP-05: Bổ sung nhánh State Transition còn thiếu. Cần trigger Batch thủ công hoặc mock date trên môi trường test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>US01-BR-HAP-014</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>LOG-SPDV-EDIT</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Mục "Khai báo Sản phẩm, dịch vụ chi tiết" - P31-P34: Chỉnh sửa SPDV chi tiết</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>SA - Tham Số Hệ Thống</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Khai báo Danh mục Sản phẩm Dịch vụ và Code Phí</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Chỉnh sửa SPDV chi tiết thành công – Sửa Ngày hiệu lực và Ngày hết hiệu lực hợp lệ</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>TC-BR</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>1. Nghiệp vụ 'Tài Khoản' (Mã '01') đã duyệt: Ngày HLực = 01/04/2026; Ngày HHLực = 31/12/2027.
+2. SPDV '0101 - TK Thanh Toán' đã duyệt, Hoạt động: Ngày HLực = 10/04/2026; Ngày HHLực = 30/06/2027.
+3. Không có SPDV cấp con nào của '0101'.
+4. Đã đăng nhập Maker. Ngày hệ thống (T) = 21/04/2026.</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>1. Truy cập menu: Tham số &gt;&gt; Danh mục sản phẩm dịch vụ và Code phí.
+2. Tại dòng '0101 - TK Thanh Toán', nhấn 'Chỉnh sửa'.
+3. Sửa Ngày hiệu lực từ 10/04/2026 → 21/04/2026 (&gt;= T ✓, &gt;= HLực cha 01/04/2026 ✓).
+4. Sửa Ngày hết hiệu lực từ 30/06/2027 → 31/10/2027 (&lt;= HHLực cha 31/12/2027 ✓).
+5. Nhấn 'Xác nhận'.</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>(i) Nghiệp vụ/Logic: Tất cả ràng buộc hợp lệ. Bản ghi Sửa SPDV tạo thành công ở trạng thái Chờ duyệt.
+(ii) UI: Toast thành công: 'Yêu cầu Sửa SPDV chi tiết đã được gửi chờ phê duyệt'. Trên lưới chính, thông tin '0101' vẫn hiển thị theo giá trị cũ cho đến khi Checker duyệt.
+(iii) Trạng thái bản ghi: Bản ghi Pending 'Sửa SPDV - 0101' xuất hiện trong Tác vụ Pending của Maker và Tác vụ chờ duyệt của Checker.
+(iv) Output: Bản ghi trong danh sách Tác vụ chờ duyệt của Checker.</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>US01-SPDV-EDIT-HAP</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Review GAP-06: Bổ sung happy path Edit SPDV chi tiết bị thiếu hoàn toàn trong bộ TC gốc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>US01-BR-NEG-014</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>LOG-SPDV-EDIT</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Mục "Khai báo Sản phẩm, dịch vụ chi tiết" - P32: "Ngày HLực cha &lt;= Ngày HLực con"; P33: "Ngày HHLực cha &gt;= Ngày HHLực con"</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>SA - Tham Số Hệ Thống</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Khai báo Danh mục Sản phẩm Dịch vụ và Code Phí</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Chỉnh sửa SPDV chi tiết thất bại – Ngày hiệu lực mới nhỏ hơn Ngày hiệu lực của cấp cha</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>TC-BR</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>1. Nghiệp vụ 'Tài Khoản' (Mã '01') đã duyệt: Ngày HLực = 15/04/2026; Ngày HHLực = 31/12/2027.
+2. SPDV '0101 - TK Thanh Toán' đã duyệt, Hoạt động: Ngày HLực = 15/04/2026; Ngày HHLực = 30/06/2027.
+3. Đã đăng nhập Maker. Ngày hệ thống (T) = 21/04/2026.</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>1. Truy cập menu: Tham số &gt;&gt; Danh mục sản phẩm dịch vụ và Code phí.
+2. Tại dòng '0101 - TK Thanh Toán', nhấn 'Chỉnh sửa'.
+3. Sửa Ngày hiệu lực từ 15/04/2026 → 21/04/2026 (&gt;= T ✓) nhưng thử nhập 10/04/2026.
+4. Nhập Ngày hiệu lực = 10/04/2026 (&lt; Ngày HLực cha = 15/04/2026 ✗).
+5. Giữ nguyên Ngày hết hiệu lực = 30/06/2027.
+6. Nhấn 'Xác nhận'.</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>(i) Nghiệp vụ/Logic: Hệ thống từ chối vì Ngày HLực mới (10/04/2026) &lt; Ngày HLực cấp cha '01' (15/04/2026). Vi phạm ràng buộc P32.
+(ii) UI: Thông báo lỗi tại trường Ngày hiệu lực: 'Ngày hiệu lực phải lớn hơn hoặc bằng Ngày hiệu lực của cấp cha (15/04/2026)'. Form vẫn mở.
+(iii) Trạng thái bản ghi: Không tạo bản ghi Pending. SPDV '0101' giữ nguyên HLực = 15/04/2026.
+(iv) Output: Không.</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>US01-SPDV-EDIT-NEG-HLUC</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Review GAP-06: Bổ sung Negative Edit SPDV chi tiết. Cần test thêm chiều HHLực (con &gt; HHLực cha) theo cùng pattern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>US01-BR-HAP-015</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>LOG-NV-AUTOCODE</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Mục "Khai báo Nghiệp vụ" - Bảng Table 2 - Mã Nghiệp vụ: "số tự tăng bắt đầu từ 01 đến 99"</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>SA - Tham Số Hệ Thống</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Khai báo Danh mục Sản phẩm Dịch vụ và Code Phí</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Thêm mới Nghiệp vụ thành công – BVA boundary last-valid: Hệ thống đã có 98 NV, tạo mới sinh Mã '99'</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>TC-BR</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>1. Đã đăng nhập với tài khoản Maker có quyền 'Danh mục Sản phẩm Dịch vụ và Code Phí'.
+2. Hệ thống đã có đúng 98 Nghiệp vụ (Mã 01→98 tồn tại, ở trạng thái bất kỳ).
+3. Ngày hệ thống (T) = 21/04/2026.</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>1. Truy cập menu: Tham số &gt;&gt; Danh mục sản phẩm dịch vụ và Code phí.
+2. Nhấn nút 'Thêm mới Nghiệp vụ'.
+3. Quan sát trường 'Mã Nghiệp vụ' trên màn hình (phải hiển thị '99').
+4. Nhập Tên Nghiệp vụ = 'NghiepVu_Last', Mô tả = 'Test BVA mã tự sinh cuối cùng hợp lệ'.
+5. Nhập Ngày hiệu lực = 21/04/2026, Ngày hết hiệu lực = 31/12/2026.
+6. Nhấn 'Xác nhận'.</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>(i) Nghiệp vụ/Logic: Hệ thống tự sinh Mã = '99' (số hợp lệ cuối cùng trong dải 01-99). Bản ghi lưu thành công ở trạng thái Chờ duyệt.
+(ii) UI: Trường Mã Nghiệp vụ hiển thị '99' (read-only). Toast thành công: 'Thêm mới Nghiệp vụ thành công'.
+(iii) Trạng thái bản ghi: Bản ghi 'NghiepVu_Last' (Mã '99') xuất hiện trong Tác vụ Pending của Maker với Action = 'Thêm mới', Status = 'Chờ duyệt'.
+(iv) Output: Bản ghi trong danh sách Tác vụ chờ duyệt của Checker.</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>US01-NV-AUTOCODE-BVA-99</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Review GAP-07: Bổ sung BVA boundary last-valid (98→99) bị thiếu. Pair với NEG-001 (99→100 overflow) để phủ đủ boundary.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>US01-BR-NEG-015</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>LOG-NV-REQUIRED-FIELDS</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Mục "Giao diện - Khai báo Nghiệp vụ" - Bảng Table 2: trường Mô tả - ký hiệu "◎" (bắt buộc)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>SA - Tham Số Hệ Thống</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Khai báo Danh mục Sản phẩm Dịch vụ và Code Phí</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Thêm mới Nghiệp vụ thất bại – Bỏ trống trường Mô tả (bắt buộc nhập)</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>TC-BR</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>1. Đã đăng nhập với tài khoản Maker có quyền 'Danh mục Sản phẩm Dịch vụ và Code Phí'.
+2. Ngày hệ thống (T) = 21/04/2026.</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>1. Truy cập menu: Tham số &gt;&gt; Danh mục sản phẩm dịch vụ và Code phí &gt;&gt; Thêm mới Nghiệp vụ.
+2. Nhập Tên Nghiệp vụ = 'Chứng Khoán'.
+3. Để trống trường Mô tả (không nhập gì).
+4. Nhập Ngày hiệu lực = 21/04/2026, Ngày hết hiệu lực = 31/12/2026.
+5. Nhấn 'Xác nhận'.</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>(i) Nghiệp vụ/Logic: Hệ thống từ chối lưu vì trường Mô tả bắt buộc nhập (ký hiệu ◎ trong Table 2).
+(ii) UI: Hiển thị thông báo lỗi tại trường Mô tả: 'Mô tả là trường bắt buộc, vui lòng nhập thông tin'. Trường Mô tả được highlight lỗi (viền đỏ hoặc tương đương). Form không đóng.
+(iii) Trạng thái bản ghi: Không có bản ghi nào được tạo.
+(iv) Output: Không.</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>US01-NV-REQUIRED-MOTA</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Review GAP-01: PENDING BA CONFIRM – Cần BA xác nhận trường Mô tả có bắt buộc không (ký hiệu ◎ trong Table 2). Nếu không bắt buộc → Skip TC này.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:U34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3536,7 +4104,7 @@
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>40</t>
         </is>
       </c>
     </row>
@@ -3548,7 +4116,7 @@
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
     </row>
@@ -3560,7 +4128,7 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>15</t>
         </is>
       </c>
     </row>
@@ -3605,10 +4173,8 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
+      <c r="B16" s="13" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
@@ -3617,10 +4183,8 @@
           <t>High</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
+      <c r="B17" s="13" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
@@ -3629,10 +4193,8 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B18" s="13" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">

</xml_diff>